<commit_message>
Refresh AI circular financing site (2026-10-09 19:58)
</commit_message>
<xml_diff>
--- a/ai_circular_financing.xlsx
+++ b/ai_circular_financing.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SpaceX -&gt; Nvidia purchase $40bn; Nvidia -&gt; SpaceX investment</t>
+          <t>SpaceX / xAI -&gt; Nvidia purchase $40bn; Nvidia -&gt; SpaceX / xAI investment</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Google -&gt; SpaceX purchase $30bn</t>
+          <t>Google -&gt; SpaceX / xAI purchase $30bn</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; SpaceX purchase $40bn</t>
+          <t>Anthropic -&gt; SpaceX / xAI purchase $40bn</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; xAI investment $2bn; xAI -&gt; Nvidia purchase $12.5bn</t>
+          <t>Nvidia -&gt; SpaceX / xAI investment $2bn; SpaceX / xAI -&gt; Nvidia purchase $12.5bn</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; xAI investment; AMD -&gt; xAI investment; xAI -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; SpaceX / xAI investment; AMD -&gt; SpaceX / xAI investment; SpaceX / xAI -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -9869,7 +9869,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>SpaceX</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -11009,7 +11009,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>SpaceX</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -12077,7 +12077,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>SpaceX</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>SpaceX</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">

</xml_diff>

<commit_message>
Refresh AI circular financing site (2026-10-15 16:39)
</commit_message>
<xml_diff>
--- a/ai_circular_financing.xlsx
+++ b/ai_circular_financing.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -492,30 +492,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Broadcom arranging over $50bn of financing for OpenAI's custom chips</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>50</v>
+          <t>Anthropic signs an unannounced multiyear cloud deal with Nvidia-backed IREN</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>WSJ report; talks</t>
+          <t>The Information report; value and term undisclosed</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Broadcom -&gt; OpenAI credit $50bn; OpenAI -&gt; Broadcom purchase</t>
+          <t>Anthropic -&gt; IREN purchase</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -535,32 +532,29 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNYy1WWHZ</t>
+          <t>https://dataconomy.com/2026/10/12/anthropic-reportedly-signs-multiyear-cloud-deal-with-iren/ | https://www.investing.com/news/stock-market-news/iren-stock-jumps-on-multiyear-cloud-deal-with-anthropic-93CH-4943757</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SpaceX seeks $40bn of Apollo-led debt to buy Nvidia chips; Nvidia is a SpaceX shareholder</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>40</v>
+          <t>Nvidia in talks to deepen its Reflection AI stake, supply more chips, or buy it</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FT report; ~$10bn loans + $30bn investment-grade debt, closing 2027</t>
+          <t>FT/Bloomberg/Reuters reports; early talks; Nvidia led Reflection's $2bn round with ~$800m (Oct 2025)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SpaceX / xAI -&gt; Nvidia purchase $40bn; Nvidia -&gt; SpaceX / xAI investment</t>
+          <t>Nvidia -&gt; Reflection AI investment; Reflection AI -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -575,7 +569,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -585,32 +579,32 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://investinglive.com/stocks/spacex-seeks-40-billion-in-debt-led-by-apollo-to-fund-nvidia-chip-order-ft-says/</t>
+          <t>https://qz.com/nvidia-reflection-ai-acquisition-investment-talks-101226 | https://finance.yahoo.com/technology/ai/articles/nvidia-talks-acquire-invest-further-111913214.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nvidia adds $1.5bn SB Energy placement at the IPO price (total $3bn)</t>
+          <t>Broadcom arranging over $50bn of financing for OpenAI's custom chips</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.5</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>prepaid at a discount; IPO delayed in Sep-Oct 2026</t>
+          <t>WSJ report (&gt;$50bn); Bloomberg 8 Oct: early talks, ~$30bn of debt for the next leg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; SB Energy investment $1.5bn</t>
+          <t>Broadcom -&gt; OpenAI credit $50bn; OpenAI -&gt; Broadcom purchase</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -620,7 +614,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -635,37 +629,37 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://energynow.com/2026/09/nvidia-buying-an-additional-1-5-billion-in-sb-energy-shares-ahead-of-ipo/</t>
+          <t>https://finance.yahoo.com/technology/ai/articles/broadcom-holds-early-talks-financing-230717190.html | https://news.bloomberglaw.com/artificial-intelligence/broadcom-holds-early-talks-about-financing-deal-for-openai-chips</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Anthropic signs $35bn Lambda deal at Hut 8's Texas site; Nvidia holds the lease</t>
+          <t>Nvidia discusses investing another $1bn in Figure AI</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Reuters / WSJ</t>
+          <t>The Information report; ~$38bn pre-money; no agreement announced</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Lambda purchase $35bn; Nvidia -&gt; Hut 8 backstop</t>
+          <t>Nvidia -&gt; Figure AI investment $1bn</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -675,7 +669,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -685,32 +679,32 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.eweek.com/news/nvidia-figure-ai-1-billion-investment-humanoid-robots/ | https://cryptobriefing.com/nvidia-discusses-1-billion-figure-ai-investment/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SB Energy gives OpenAI ~$5.5bn of warrants; OpenAI invests $500m and SB Energy buys OpenAI services</t>
+          <t>SpaceX seeks $40bn of Apollo-led debt to buy Nvidia chips; Nvidia is a SpaceX shareholder</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>WSJ</t>
+          <t>FT report; ~$10bn loans + $30bn investment-grade debt, closing 2027</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SB Energy -&gt; OpenAI stock_grant $5.5bn; OpenAI -&gt; SB Energy investment $0.5bn; SB Energy -&gt; OpenAI purchase</t>
+          <t>SpaceX / xAI -&gt; Nvidia purchase $40bn; Nvidia -&gt; SpaceX / xAI investment</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -735,47 +729,47 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://investinglive.com/stocks/spacex-seeks-40-billion-in-debt-led-by-apollo-to-fund-nvidia-chip-order-ft-says/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Anthropic signs $45bn, 6-year Nscale contract in West Virginia</t>
+          <t>Qualcomm gives Amazon warrants worth up to $4bn tied to AI data-centre chip purchases</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FT report</t>
+          <t>25m shares at $161.26, vesting with purchases of up to $60bn; expire Sep 2036</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Nscale purchase $45bn</t>
+          <t>Qualcomm -&gt; Amazon stock_grant $4bn; Amazon -&gt; Qualcomm purchase</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -785,32 +779,32 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://finance.yahoo.com/technology/ai/articles/qualcomm-ai-ambitions-boost-amazon-151217166.html | https://www.tradingpedia.com/2026/09/10/qualcomm-gives-amazon-multi-billion-dollar-ai-chip-warrant/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Marvell gives Google warrants worth up to $12.2bn tied to custom-chip purchases</t>
+          <t>Nscale sells Figure AI $3.5bn of compute and takes an equity stake</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12.2</v>
+        <v>3.5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>58.97m shares at $206.58; one tranche vests per $500m of Google purchases (ceiling $120bn)</t>
+          <t>intent to scale past $6bn; Nvidia is an investor in both</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Marvell -&gt; Google stock_grant $12.2bn; Google -&gt; Marvell purchase</t>
+          <t>Nscale -&gt; Figure AI investment; Figure AI -&gt; Nscale purchase $3.5bn</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -820,7 +814,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -835,32 +829,32 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.vktr.com/ai-news/marvell-gives-google-option-to-buy-122-billion-stake-in-custom-ai-chip-deal/</t>
+          <t>https://www.nscale.com/press-releases/nscale-and-figure | https://thenextweb.com/news/nscale-figure-3-5bn-compute-equity-stake</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nvidia guarantees up to $105bn for OpenAI's 8 GW Ohio campus and invests $1.5bn in SB Energy</t>
+          <t>Nvidia adds $1.5bn SB Energy placement at the IPO price (total $3bn)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>106.5</v>
+        <v>1.5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RVG cap from Nvidia filing; first 800 MW in 2028</t>
+          <t>prepaid at a discount; IPO delayed in Sep-Oct 2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; SB Energy backstop $105bn; Nvidia -&gt; SB Energy investment $1.5bn; OpenAI -&gt; SB Energy purchase; SB Energy -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; SB Energy investment $1.5bn</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -875,7 +869,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -885,32 +879,32 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://pulse2.com/nvidia-invests-1-5-billion-in-sb-energy-and-backs-8-gw-openai-ai-factory-campus-in-ohio | https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001045810&amp;type=10-Q</t>
+          <t>https://energynow.com/2026/09/nvidia-buying-an-additional-1-5-billion-in-sb-energy-shares-ahead-of-ipo/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nvidia and six financiers target $500bn of AI compute financing; Nvidia offers residual-value support</t>
+          <t>Anthropic signs $35bn Lambda deal at Hut 8's Texas site; Nvidia holds the lease</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>500</v>
+        <v>35</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>non-binding MOUs; Nvidia support up to 25% of each project; not summed</t>
+          <t>Reuters / WSJ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; AI compute financing platforms backstop; Apollo -&gt; AI compute financing platforms credit</t>
+          <t>Anthropic -&gt; Lambda purchase $35bn; Nvidia -&gt; Hut 8 backstop</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -920,57 +914,57 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://blogs.nvidia.com/blog/nvidia-ai-factory-compute/ | https://www.ft.com/content/9a6947bf-9d4e-4489-80b9-2178ea657a67</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nvidia in talks to guarantee ~$250bn of OpenAI's Ohio data-centre financing</t>
+          <t>SB Energy gives OpenAI ~$5.5bn of warrants; OpenAI invests $500m and SB Energy buys OpenAI services</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>250</v>
+        <v>6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>WSJ; plus talks on up to $350bn of chip financing. Signed 17 Aug as an up-to-$105bn guarantee - not summed</t>
+          <t>WSJ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; OpenAI backstop $250bn</t>
+          <t>SB Energy -&gt; OpenAI stock_grant $5.5bn; OpenAI -&gt; SB Energy investment $0.5bn; SB Energy -&gt; OpenAI purchase</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>superseded: signed 17 Aug 2026 as up-to-$105bn RVG</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -980,52 +974,52 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://thenextweb.com/news/nvidia-openai-250bn-data-centre-financing-guarantee</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AMD to invest up to $5bn in Anthropic as Anthropic deploys 2 GW of AMD GPUs</t>
+          <t>Anthropic signs $45bn, 6-year Nscale contract in West Virginia</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>up to</t>
+          <t>FT report</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AMD -&gt; Anthropic investment $5bn; Anthropic -&gt; AMD purchase</t>
+          <t>Anthropic -&gt; Nscale purchase $45bn</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1042,26 +1036,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Anthropic signs $19bn, 20-year lease at TeraWulf's Kentucky campus</t>
+          <t>Marvell gives Google warrants worth up to $12.2bn tied to custom-chip purchases</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>12.2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>58.97m shares at $206.58; one tranche vests per $500m of Google purchases (ceiling $120bn)</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; TeraWulf purchase $19bn</t>
+          <t>Marvell -&gt; Google stock_grant $12.2bn; Google -&gt; Marvell purchase</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1081,34 +1079,37 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.vktr.com/ai-news/marvell-gives-google-option-to-buy-122-billion-stake-in-custom-ai-chip-deal/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Micron invests in Anthropic and signs supply agreement</t>
-        </is>
+          <t>Nvidia guarantees up to $105bn for OpenAI's 8 GW Ohio campus and invests $1.5bn in SB Energy</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>106.5</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>amount not disclosed</t>
+          <t>RVG cap from Nvidia filing; first 800 MW in 2028</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Micron -&gt; Anthropic investment; Micron -&gt; Anthropic purchase; Anthropic -&gt; Micron purchase</t>
+          <t>Nvidia -&gt; SB Energy backstop $105bn; Nvidia -&gt; SB Energy investment $1.5bn; OpenAI -&gt; SB Energy purchase; SB Energy -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1128,32 +1129,32 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://pulse2.com/nvidia-invests-1-5-billion-in-sb-energy-and-backs-8-gw-openai-ai-factory-campus-in-ohio | https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001045810&amp;type=10-Q</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Broadcom, Apollo and Blackstone set up $35bn chip-lease vehicle for Anthropic</t>
+          <t>Nvidia and six financiers target $500bn of AI compute financing; Nvidia offers residual-value support</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>500</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Broadcom sells TPUs to the vehicle and backstops most of its debt; Apollo/Blackstone completed the $35bn in Oct 2026, package reportedly expanding toward $60bn</t>
+          <t>non-binding MOUs; Nvidia support up to 25% of each project; not summed</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Broadcom -&gt; Anthropic backstop $35bn; Anthropic -&gt; Broadcom purchase</t>
+          <t>Nvidia -&gt; AI compute financing platforms backstop; Apollo -&gt; AI compute financing platforms credit</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1163,112 +1164,112 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a | https://www.ft.com/content/9a6947bf-9d4e-4489-80b9-2178ea657a67</t>
+          <t>https://blogs.nvidia.com/blog/nvidia-ai-factory-compute/ | https://www.ft.com/content/9a6947bf-9d4e-4489-80b9-2178ea657a67</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Google pays SpaceX ~$30bn for xAI's Colossus compute</t>
+          <t>Nvidia in talks to guarantee ~$250bn of OpenAI's Ohio data-centre financing</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>$920m a month for ~110,000 Nvidia GPUs, Oct 2026 to Jun 2029 (SpaceX SEC filing)</t>
+          <t>WSJ; plus talks on up to $350bn of chip financing. Signed 17 Aug as an up-to-$105bn guarantee - not summed</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Google -&gt; SpaceX / xAI purchase $30bn</t>
+          <t>Nvidia -&gt; OpenAI backstop $250bn</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>superseded: signed 17 Aug 2026 as up-to-$105bn RVG</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://news.bloomberglaw.com/mergers-and-acquisitions/spacex-inks-30-billion-computing-power-deal-with-google-1</t>
+          <t>https://thenextweb.com/news/nvidia-openai-250bn-data-centre-financing-guarantee</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Anthropic to pay SpaceX/xAI ~$40bn for Colossus compute</t>
+          <t>AMD to invest up to $5bn in Anthropic as Anthropic deploys 2 GW of AMD GPUs</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>through May 2029 (reported)</t>
+          <t>up to</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; SpaceX / xAI purchase $40bn</t>
+          <t>AMD -&gt; Anthropic investment $5bn; Anthropic -&gt; AMD purchase</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1285,31 +1286,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nvidia to invest up to $2.1bn in IREN and rent $3.4bn of its capacity</t>
+          <t>Anthropic signs $19bn, 20-year lease at TeraWulf's Kentucky campus</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.5</v>
+        <v>19</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; IREN investment $2.1bn; Nvidia -&gt; IREN purchase $3.4bn; IREN -&gt; Nvidia purchase</t>
+          <t>Anthropic -&gt; TeraWulf purchase $19bn</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1324,37 +1325,34 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-05-07/nvidia-to-invest-up-to-2-1-billion-in-data-center-firm-iren</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nvidia takes rights to invest up to $3.2bn in Corning to fund optical plants</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>3.2</v>
+          <t>Micron invests in Anthropic and signs supply agreement</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>up to</t>
+          <t>amount not disclosed</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Corning investment $3.2bn; Nvidia -&gt; Corning purchase</t>
+          <t>Micron -&gt; Anthropic investment; Micron -&gt; Anthropic purchase; Anthropic -&gt; Micron purchase</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1374,42 +1372,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/sectors/technology/articles/nvidia-expands-ai-investment-push-213531266.html</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Google invests $10bn (up to $40bn) in Anthropic; 5 GW of TPUs</t>
+          <t>Broadcom, Apollo and Blackstone set up $35bn chip-lease vehicle for Anthropic</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>$10bn at $350bn valuation + up to $30bn on milestones</t>
+          <t>Broadcom sells TPUs to the vehicle and backstops most of its debt; Apollo/Blackstone completed the $35bn in Oct 2026, package reportedly expanding toward $60bn; Anthropic IPO filing (1 Oct 2026): Broadcom to lend up to $42bn, possibly convertible; Bloomberg (2 Oct): $60bn package = $42bn senior + $18bn junior, syndicating Oct</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Google -&gt; Anthropic investment $40bn; Anthropic -&gt; Google purchase</t>
+          <t>Broadcom -&gt; Anthropic backstop $35bn; Anthropic -&gt; Broadcom purchase</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1424,47 +1422,47 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://cybernews.com/ai-news/google-to-invest-up-to-40b-in-anthropic-as-ai-rivalry-accelerates/</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a | https://www.ft.com/content/9a6947bf-9d4e-4489-80b9-2178ea657a67 | https://www.cnbc.com/2026/10/01/broadcom-lending-anthropic-42-billion-chips-reuters.html | https://www.bloomberg.com/news/articles/2026-10-02/broadcom-starts-amassing-60-billion-to-fund-chips-for-anthropic | https://www.ifre.com/loans/2496132/chips-with-everything-broadcom-backstops-us42bn-funding-for-anthropic</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Amazon invests up to $25bn more in Anthropic; Anthropic commits $100bn+ to AWS</t>
+          <t>Google pays SpaceX ~$30bn for xAI's Colossus compute</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>$5bn now, $20bn on milestones; AWS spend through 2036</t>
+          <t>$920m a month for ~110,000 Nvidia GPUs, Oct 2026 to Jun 2029 (SpaceX SEC filing)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Amazon -&gt; Anthropic investment $25bn; Anthropic -&gt; Amazon purchase $100bn</t>
+          <t>Google -&gt; SpaceX / xAI purchase $30bn</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1474,29 +1472,32 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://thenextweb.com/news/amazon-anthropic-25-billion-investment | https://www.anthropic.com/news/anthropic-amazon-compute</t>
+          <t>https://news.bloomberglaw.com/mergers-and-acquisitions/spacex-inks-30-billion-computing-power-deal-with-google-1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CoreWeave to supply Claude compute from late 2026</t>
-        </is>
+          <t>Anthropic to pay SpaceX/xAI ~$40bn for Colossus compute</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>40</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>value not disclosed</t>
+          <t>through May 2029 (reported)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; CoreWeave purchase</t>
+          <t>Anthropic -&gt; SpaceX / xAI purchase $40bn</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1506,12 +1507,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1528,27 +1529,26 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Anthropic secures multiple GW of Google/Broadcom TPU capacity from 2027</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>value not disclosed</t>
-        </is>
-      </c>
+          <t>Nvidia to invest up to $2.1bn in IREN and rent $3.4bn of its capacity</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Google purchase; Anthropic -&gt; Broadcom purchase</t>
+          <t>Nvidia -&gt; IREN investment $2.1bn; Nvidia -&gt; IREN purchase $3.4bn; IREN -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1568,42 +1568,42 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.bloomberg.com/news/articles/2026-05-07/nvidia-to-invest-up-to-2-1-billion-in-data-center-firm-iren</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Amazon invests $50bn in OpenAI; OpenAI adds $100bn to its AWS contract</t>
+          <t>Nvidia takes rights to invest up to $3.2bn in Corning to fund optical plants</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>150</v>
+        <v>3.2</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>$15bn upfront, $35bn conditional on IPO or AGI; round closed 31 Mar at $852bn</t>
+          <t>up to</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Amazon -&gt; OpenAI investment $50bn; OpenAI -&gt; Amazon purchase $100bn</t>
+          <t>Nvidia -&gt; Corning investment $3.2bn; Nvidia -&gt; Corning purchase</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1618,47 +1618,47 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/markets/stocks/articles/openai-closes-122bn-funding-round-093126735.html | https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://finance.yahoo.com/sectors/technology/articles/nvidia-expands-ai-investment-push-213531266.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nvidia invests $30bn in OpenAI's $122bn round</t>
+          <t>Google invests $10bn (up to $40bn) in Anthropic; 5 GW of TPUs</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>replaces the 2025 LOI; not tied to deployment milestones</t>
+          <t>$10bn at $350bn valuation + up to $30bn on milestones</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; OpenAI investment $30bn; OpenAI -&gt; Nvidia purchase</t>
+          <t>Google -&gt; Anthropic investment $40bn; Anthropic -&gt; Google purchase</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1668,28 +1668,32 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.outlookbusiness.com/corporate/nvidia-to-invest-30bn-in-openai-previous-100bn-partnership-plan-scrapped</t>
+          <t>https://cybernews.com/ai-news/google-to-invest-up-to-40b-in-anthropic-as-ai-rivalry-accelerates/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SoftBank invests $30bn in OpenAI's $122bn round</t>
+          <t>Amazon invests up to $25bn more in Anthropic; Anthropic commits $100bn+ to AWS</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>125</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>$5bn now, $20bn on milestones; AWS spend through 2036</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SoftBank -&gt; OpenAI investment $30bn</t>
+          <t>Amazon -&gt; Anthropic investment $25bn; Anthropic -&gt; Amazon purchase $100bn</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1699,12 +1703,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1714,37 +1718,34 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/markets/stocks/articles/openai-closes-122bn-funding-round-093126735.html</t>
+          <t>https://thenextweb.com/news/amazon-anthropic-25-billion-investment | https://www.anthropic.com/news/anthropic-amazon-compute</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AMD gives Meta warrants for up to 10% of AMD as Meta commits to 6 GW of AMD GPUs</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>60</v>
+          <t>CoreWeave to supply Claude compute from late 2026</t>
+        </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>reported $60bn to &gt;$100bn</t>
+          <t>value not disclosed</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Meta -&gt; AMD purchase $60bn; AMD -&gt; Meta stock_grant</t>
+          <t>Anthropic -&gt; CoreWeave purchase</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1754,7 +1755,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1764,47 +1765,44 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://roic.ai/news/meta-strikes-60-billion-ai-chip-mega-deal-with-amd-securing-6-gigawatts-and-potential-stake-02-24-2026 | https://ny1.com/nyc/all-boroughs/ap-top-news/2026/02/24/facebook-owner-meta-to-buy-ai-chips-from-amd-in-deal-worth-up-to-100-billion</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AMD backstops a $300m Goldman loan so Crusoe can buy AMD chips</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0.3</v>
+          <t>Anthropic secures multiple GW of Google/Broadcom TPU capacity from 2027</t>
+        </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>loan secured on the chips; AMD will rent them back if Crusoe finds no customers (The Information)</t>
+          <t>value not disclosed</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AMD -&gt; Crusoe backstop $0.3bn; Crusoe -&gt; AMD purchase $0.3bn</t>
+          <t>Anthropic -&gt; Google purchase; Anthropic -&gt; Broadcom purchase</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1814,33 +1812,37 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/amd-underwrites-300m-crusoe-loan-so-data-center-firm-can-buy-its-ai-chips-report/</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nvidia invests another $2bn in CoreWeave</t>
+          <t>Amazon invests $50bn in OpenAI; OpenAI adds $100bn to its AWS contract</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
-      </c>
-      <c r="D29" t="inlineStr"/>
+        <v>150</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>$15bn upfront, $35bn conditional on IPO or AGI; round closed 31 Mar at $852bn</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; CoreWeave investment $2bn; CoreWeave -&gt; Nvidia purchase</t>
+          <t>Amazon -&gt; OpenAI investment $50bn; OpenAI -&gt; Amazon purchase $100bn</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1860,47 +1862,47 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://finance.yahoo.com/markets/stocks/articles/openai-closes-122bn-funding-round-093126735.html | https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>OpenAI signs &gt;$10bn, 750 MW compute deal with Cerebras</t>
+          <t>Nvidia invests $30bn in OpenAI's $122bn round</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>reported floor</t>
+          <t>replaces the 2025 LOI; not tied to deployment milestones</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; Cerebras purchase $10bn</t>
+          <t>Nvidia -&gt; OpenAI investment $30bn; OpenAI -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1910,37 +1912,33 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.outlookbusiness.com/corporate/nvidia-to-invest-30bn-in-openai-previous-100bn-partnership-plan-scrapped</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>xAI raises $20bn Series E with Nvidia; GPU SPV leases chips to xAI</t>
+          <t>SoftBank invests $30bn in OpenAI's $122bn round</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>20</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>~$7.5bn equity + up to $12.5bn SPV debt (Bloomberg); Nvidia up to ~$2bn reported</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; SpaceX / xAI investment $2bn; SpaceX / xAI -&gt; Nvidia purchase $12.5bn</t>
+          <t>SoftBank -&gt; OpenAI investment $30bn</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1950,7 +1948,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1960,47 +1958,47 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://pulse2.com/xai-20-billion-series-e-funding/ | https://www.outlookbusiness.com/artificial-intelligence/elon-musks-xai-raises-20-bn-in-series-e-round-backed-by-nvidia</t>
+          <t>https://finance.yahoo.com/markets/stocks/articles/openai-closes-122bn-funding-round-093126735.html | https://www.konsulteer.com/article/softbank-completes-30-billion-openai-investment-bringing-total-commitment-to-64-6-billion</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Broadcom books $21bn of TPU rack orders from Anthropic</t>
+          <t>AMD gives Meta warrants for up to 10% of AMD as Meta commits to 6 GW of AMD GPUs</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>$10bn (Sep) + $11bn (Dec) orders</t>
+          <t>reported $60bn to &gt;$100bn</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Broadcom purchase $21bn</t>
+          <t>Meta -&gt; AMD purchase $60bn; AMD -&gt; Meta stock_grant</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2010,43 +2008,47 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://investors.broadcom.com/news-releases</t>
+          <t>https://roic.ai/news/meta-strikes-60-billion-ai-chip-mega-deal-with-amd-securing-6-gigawatts-and-potential-stake-02-24-2026 | https://ny1.com/nyc/all-boroughs/ap-top-news/2026/02/24/facebook-owner-meta-to-buy-ai-chips-from-amd-in-deal-worth-up-to-100-billion</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nvidia invests $2bn in Synopsys</t>
+          <t>AMD backstops a $300m Goldman loan so Crusoe can buy AMD chips</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" t="inlineStr"/>
+        <v>0.3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>loan secured on the chips; AMD will rent them back if Crusoe finds no customers (The Information)</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Synopsys investment $2bn; Synopsys -&gt; Nvidia purchase</t>
+          <t>AMD -&gt; Crusoe backstop $0.3bn; Crusoe -&gt; AMD purchase $0.3bn</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2056,38 +2058,38 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-and-synopsys-announce-strategic-partnership</t>
+          <t>https://www.datacenterdynamics.com/en/news/amd-underwrites-300m-crusoe-loan-so-data-center-firm-can-buy-its-ai-chips-report/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Microsoft (up to $5bn) and Nvidia (up to $10bn) invest in Anthropic; Anthropic buys $30bn of Azure</t>
+          <t>Nvidia invests another $2bn in CoreWeave</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Anthropic investment $5bn; Nvidia -&gt; Anthropic investment $10bn; Anthropic -&gt; Microsoft purchase $30bn; Anthropic -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; CoreWeave investment $2bn; CoreWeave -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2102,32 +2104,32 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/microsoft-nvidia-anthropic-announce-strategic-partnerships</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Anthropic plans $50bn of US data centres with Fluidstack</t>
+          <t>OpenAI signs &gt;$10bn, 750 MW compute deal with Cerebras</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>multi-site plan; may overlap the TeraWulf and Cipher leases</t>
+          <t>reported floor</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Fluidstack purchase $50bn</t>
+          <t>OpenAI -&gt; Cerebras purchase $10bn</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2142,7 +2144,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2152,37 +2154,37 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/anthropic-invests-50-billion-in-american-ai-infrastructure</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Meta signs $3bn contract with Nebius</t>
+          <t>xAI raises $20bn Series E with Nvidia; GPU SPV leases chips to xAI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5 years</t>
+          <t>~$7.5bn equity + up to $12.5bn SPV debt (Bloomberg); Nvidia up to ~$2bn reported</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Meta -&gt; Nebius purchase $3bn</t>
+          <t>Nvidia -&gt; SpaceX / xAI investment $2bn; SpaceX / xAI -&gt; Nvidia purchase $12.5bn</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2192,7 +2194,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2202,33 +2204,37 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://nebius.com/newsroom</t>
+          <t>https://pulse2.com/xai-20-billion-series-e-funding/ | https://www.outlookbusiness.com/artificial-intelligence/elon-musks-xai-raises-20-bn-in-series-e-round-backed-by-nvidia</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-11-03</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>OpenAI signs $38bn, 7-year AWS contract</t>
+          <t>Broadcom books $21bn of TPU rack orders from Anthropic</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>38</v>
-      </c>
-      <c r="D37" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>$10bn (Sep) + $11bn (Dec) orders</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; Amazon purchase $38bn</t>
+          <t>Anthropic -&gt; Broadcom purchase $21bn</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2248,33 +2254,33 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://openai.com/index/aws-and-openai-partnership/</t>
+          <t>https://investors.broadcom.com/news-releases</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-11-03</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Microsoft signs $9.7bn, 5-year contract with IREN (20% prepaid)</t>
+          <t>Nvidia invests $2bn in Synopsys</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9.699999999999999</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; IREN purchase $9.7bn; IREN -&gt; Dell purchase $5.8bn</t>
+          <t>Nvidia -&gt; Synopsys investment $2bn; Synopsys -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2294,47 +2300,43 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://iren.com/</t>
+          <t>https://nvidianews.nvidia.com/news/nvidia-and-synopsys-announce-strategic-partnership</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nvidia to invest up to $1bn in Poolside; Poolside rents 40,000 GB300s from CoreWeave</t>
+          <t>Microsoft (up to $5bn) and Nvidia (up to $10bn) invest in Anthropic; Anthropic buys $30bn of Azure</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>up to (Bloomberg)</t>
-        </is>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Poolside investment $1bn; Poolside -&gt; CoreWeave purchase</t>
+          <t>Microsoft -&gt; Anthropic investment $5bn; Nvidia -&gt; Anthropic investment $10bn; Anthropic -&gt; Microsoft purchase $30bn; Anthropic -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2344,42 +2346,42 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.anthropic.com/news/microsoft-nvidia-anthropic-announce-strategic-partnerships</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>OpenAI recapitalisation: Microsoft keeps ~27%, OpenAI commits $250bn more to Azure</t>
+          <t>Anthropic plans $50bn of US data centres with Fluidstack</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Microsoft stake valued ~$135bn; no new cash</t>
+          <t>multi-site plan; may overlap the TeraWulf and Cipher leases</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; Microsoft purchase $250bn; Microsoft -&gt; OpenAI investment</t>
+          <t>Anthropic -&gt; Fluidstack purchase $50bn</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2394,33 +2396,37 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://blogs.microsoft.com/blog/2025/10/28/the-next-chapter-of-the-microsoft-openai-partnership/</t>
+          <t>https://www.anthropic.com/news/anthropic-invests-50-billion-in-american-ai-infrastructure</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2025-11-11</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nvidia invests $1bn in Nokia for AI-RAN</t>
+          <t>Meta signs $3bn contract with Nebius</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Nokia investment $1bn; Nokia -&gt; Nvidia purchase</t>
+          <t>Meta -&gt; Nebius purchase $3bn</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2440,29 +2446,28 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-nokia-ai-ran</t>
+          <t>https://nebius.com/newsroom</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-11-03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Anthropic to use up to 1m Google TPUs (tens of billions of dollars)</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>value not disclosed</t>
-        </is>
-      </c>
+          <t>OpenAI signs $38bn, 7-year AWS contract</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>38</v>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Anthropic -&gt; Google purchase</t>
+          <t>OpenAI -&gt; Amazon purchase $38bn</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2472,7 +2477,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2487,32 +2492,28 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/expanding-our-use-of-google-cloud-tpus-and-services</t>
+          <t>https://openai.com/index/aws-and-openai-partnership/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-11-03</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Microsoft signs ~$14bn Nscale deal for ~200,000 Nvidia GB300s</t>
+          <t>Microsoft signs $9.7bn, 5-year contract with IREN (20% prepaid)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>14</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>estimate; terms undisclosed</t>
-        </is>
-      </c>
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Nscale purchase $14bn; Nscale -&gt; Nvidia purchase</t>
+          <t>Microsoft -&gt; IREN purchase $9.7bn; IREN -&gt; Dell purchase $5.8bn</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2522,12 +2523,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2537,44 +2538,47 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/nscale-to-supply-microsoft-with-additional-100000-nvidia-gpus-in-us-and-europe/</t>
+          <t>https://iren.com/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2025-10-13</t>
+          <t>2025-10-30</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>OpenAI and Broadcom to deploy 10 GW of custom accelerators</t>
-        </is>
+          <t>Nvidia to invest up to $1bn in Poolside; Poolside rents 40,000 GB300s from CoreWeave</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>value not disclosed</t>
+          <t>up to (Bloomberg)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; Broadcom purchase</t>
+          <t>Nvidia -&gt; Poolside investment $1bn; Poolside -&gt; CoreWeave purchase</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2584,39 +2588,42 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://openai.com/index/openai-and-broadcom-announce-strategic-collaboration/</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2025-10-06</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AMD gives OpenAI warrants for up to 10% of AMD as OpenAI commits to 6 GW of AMD GPUs</t>
-        </is>
+          <t>OpenAI recapitalisation: Microsoft keeps ~27%, OpenAI commits $250bn more to Azure</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>250</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>value not disclosed; AMD says tens of billions of revenue</t>
+          <t>Microsoft stake valued ~$135bn; no new cash</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; AMD purchase; AMD -&gt; OpenAI stock_grant</t>
+          <t>OpenAI -&gt; Microsoft purchase $250bn; Microsoft -&gt; OpenAI investment</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2631,37 +2638,33 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>https://openai.com/index/openai-amd-strategic-partnership/</t>
+          <t>https://blogs.microsoft.com/blog/2025/10/28/the-next-chapter-of-the-microsoft-openai-partnership/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Meta signs $14.2bn compute contract with CoreWeave</t>
+          <t>Nvidia invests $1bn in Nokia for AI-RAN</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>through 2031</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Meta -&gt; CoreWeave purchase $14.2bn</t>
+          <t>Nvidia -&gt; Nokia investment $1bn; Nokia -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2681,38 +2684,39 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://nvidianews.nvidia.com/news/nvidia-nokia-ai-ran</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Google backstops $1.4bn of Fluidstack's Cipher lease for a 5.4% stake</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D47" t="inlineStr"/>
+          <t>Anthropic to use up to 1m Google TPUs (tens of billions of dollars)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>value not disclosed</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Google -&gt; Fluidstack backstop $1.4bn; Cipher Mining -&gt; Google stock_grant; Fluidstack -&gt; Cipher Mining purchase $3bn</t>
+          <t>Anthropic -&gt; Google purchase</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2727,28 +2731,32 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://investors.ciphermining.com/news-events/press-releases</t>
+          <t>https://www.anthropic.com/news/expanding-our-use-of-google-cloud-tpus-and-services</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>OpenAI expands CoreWeave contract by $6.5bn (total $22.4bn)</t>
+          <t>Microsoft signs ~$14bn Nscale deal for ~200,000 Nvidia GB300s</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="D48" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>estimate; terms undisclosed</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; CoreWeave purchase $6.5bn</t>
+          <t>Microsoft -&gt; Nscale purchase $14bn; Nscale -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2758,12 +2766,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2773,42 +2781,39 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://www.datacenterdynamics.com/en/news/nscale-to-supply-microsoft-with-additional-100000-nvidia-gpus-in-us-and-europe/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>2025-10-13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Nscale raises $1.1bn Series B with Nvidia, Nokia and Dell</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>1.1</v>
+          <t>OpenAI and Broadcom to deploy 10 GW of custom accelerators</t>
+        </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>round total</t>
+          <t>value not disclosed</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Nscale investment; Nscale -&gt; Nvidia purchase</t>
+          <t>OpenAI -&gt; Broadcom purchase</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2823,32 +2828,29 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://openai.com/index/openai-and-broadcom-announce-strategic-collaboration/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2025-09-22</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Nvidia to invest up to $100bn in OpenAI as it deploys 10 GW of Nvidia systems</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>100</v>
+          <t>AMD gives OpenAI warrants for up to 10% of AMD as OpenAI commits to 6 GW of AMD GPUs</t>
+        </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>LOI, $10bn per GW deployed</t>
+          <t>value not disclosed; AMD says tens of billions of revenue</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; OpenAI investment $100bn; OpenAI -&gt; Nvidia purchase</t>
+          <t>OpenAI -&gt; AMD purchase; AMD -&gt; OpenAI stock_grant</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2858,7 +2860,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>superseded: replaced by $30bn equity in Mar-2026 round</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2873,33 +2875,37 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/openai-and-nvidia-announce-strategic-partnership-to-deploy-10gw-of-nvidia-systems | https://www.business-standard.com/world-news/pledge-to-invest-100-bn-in-openai-was-never-a-commitment-nvidia-126020201582_1.html</t>
+          <t>https://openai.com/index/openai-amd-strategic-partnership/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nvidia invests $5bn in Intel and co-develops chips</t>
+          <t>Meta signs $14.2bn compute contract with CoreWeave</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>5</v>
-      </c>
-      <c r="D51" t="inlineStr"/>
+        <v>14.2</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>through 2031</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Intel investment $5bn; Intel -&gt; Nvidia purchase; Nvidia -&gt; Intel purchase</t>
+          <t>Meta -&gt; CoreWeave purchase $14.2bn</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2919,32 +2925,28 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-and-intel-to-develop-ai-infrastructure-and-personal-computing-products</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Microsoft signs ~$6.2bn Nscale/Aker contract for Stargate Norway GPUs</t>
+          <t>Google backstops $1.4bn of Fluidstack's Cipher lease for a 5.4% stake</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>5 years, ~52,000 GPUs (reported)</t>
-        </is>
-      </c>
+        <v>4.4</v>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Nscale purchase $6.2bn</t>
+          <t>Google -&gt; Fluidstack backstop $1.4bn; Cipher Mining -&gt; Google stock_grant; Fluidstack -&gt; Cipher Mining purchase $3bn</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2954,12 +2956,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2969,37 +2971,33 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://www.computing.co.uk/news/2025/nscale-strikes-14-billion-ai-deal-with-microsoft</t>
+          <t>https://investors.ciphermining.com/news-events/press-releases</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nvidia commits $6.3bn to buy CoreWeave's unused capacity</t>
+          <t>OpenAI expands CoreWeave contract by $6.5bn (total $22.4bn)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>through Apr 2032 (CoreWeave 8-K)</t>
-        </is>
-      </c>
+        <v>6.5</v>
+      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; CoreWeave backstop $6.3bn</t>
+          <t>OpenAI -&gt; CoreWeave purchase $6.5bn</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3026,25 +3024,25 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2025-09-09</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Mistral raises EUR1.7bn led by ASML, with Nvidia</t>
+          <t>Nscale raises $1.1bn Series B with Nvidia, Nokia and Dell</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>EUR1.7bn at ~1.17 USD</t>
+          <t>round total</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Mistral investment; Mistral -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; Nscale investment; Nscale -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3076,35 +3074,35 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2025-09-08</t>
+          <t>2025-09-22</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Microsoft signs $17.4bn (up to $19.4bn) GPU contract with Nebius</t>
+          <t>Nvidia to invest up to $100bn in OpenAI as it deploys 10 GW of Nvidia systems</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>19.4</v>
+        <v>100</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>up to; 5 years from Vineland, NJ</t>
+          <t>LOI, $10bn per GW deployed</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Nebius purchase $19.4bn; Nebius -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; OpenAI investment $100bn; OpenAI -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>superseded: replaced by $30bn equity in Mar-2026 round</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3119,47 +3117,43 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>https://nebius.com/newsroom/nebius-announces-multi-billion-dollar-agreement-with-microsoft-for-ai-infrastructure</t>
+          <t>https://nvidianews.nvidia.com/news/openai-and-nvidia-announce-strategic-partnership-to-deploy-10gw-of-nvidia-systems | https://www.business-standard.com/world-news/pledge-to-invest-100-bn-in-openai-was-never-a-commitment-nvidia-126020201582_1.html</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Nvidia agrees $1.5bn to rent back its own GPUs from Lambda</t>
+          <t>Nvidia invests $5bn in Intel and co-develops chips</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>$1.3bn for 10,000 GPUs + $200m for 8,000 (The Information)</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Lambda backstop $1.5bn; Lambda -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; Intel investment $5bn; Intel -&gt; Nvidia purchase; Nvidia -&gt; Intel purchase</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3169,32 +3163,32 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>https://www.theinformation.com/articles/nvidia-quietly-boosts-cloud-ally-1-5-billion-deal-rent-ai-chips</t>
+          <t>https://nvidianews.nvidia.com/news/nvidia-and-intel-to-develop-ai-infrastructure-and-personal-computing-products</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2025-08-14</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Google backstops $3.2bn of Fluidstack leases at TeraWulf for a stake</t>
+          <t>Microsoft signs ~$6.2bn Nscale/Aker contract for Stargate Norway GPUs</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6.9</v>
+        <v>6.2</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Google takes warrants for ~14% of TeraWulf after the Sept expansion</t>
+          <t>5 years, ~52,000 GPUs (reported)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Google -&gt; Fluidstack backstop $3.2bn; TeraWulf -&gt; Google stock_grant; Fluidstack -&gt; TeraWulf purchase $3.7bn</t>
+          <t>Microsoft -&gt; Nscale purchase $6.2bn</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3204,12 +3198,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3219,47 +3213,47 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>https://investors.terawulf.com/news-events/press-releases</t>
+          <t>https://www.computing.co.uk/news/2025/nscale-strikes-14-billion-ai-deal-with-microsoft</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2025-07-22</t>
+          <t>2025-09-15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>OpenAI commits ~$300bn to Oracle for 4.5 GW of Stargate capacity</t>
+          <t>Nvidia commits $6.3bn to buy CoreWeave's unused capacity</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>300</v>
+        <v>6.3</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4.5 GW confirmed; ~$300bn over ~5 years from 2027 reported (WSJ)</t>
+          <t>through Apr 2032 (CoreWeave 8-K)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; Oracle purchase $300bn</t>
+          <t>Nvidia -&gt; CoreWeave backstop $6.3bn</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3269,33 +3263,37 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://openai.com/index/stargate-advances-with-partnership-with-oracle/ | https://www.ft.com/content/86895a63-2c5b-4aea-b385-418130b64996</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-06-12</t>
+          <t>2025-09-09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Meta buys 49% of Scale AI for $14.3bn</t>
+          <t>Mistral raises EUR1.7bn led by ASML, with Nvidia</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="D59" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>EUR1.7bn at ~1.17 USD</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Meta -&gt; Scale AI investment $14.3bn; Meta -&gt; Scale AI purchase</t>
+          <t>Nvidia -&gt; Mistral investment; Mistral -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3322,25 +3320,25 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2025-05-23</t>
+          <t>2025-09-08</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Oracle to buy ~$40bn of Nvidia chips for OpenAI's Abilene site</t>
+          <t>Microsoft signs $17.4bn (up to $19.4bn) GPU contract with Nebius</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>40</v>
+        <v>19.4</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>~400,000 GB200s (FT)</t>
+          <t>up to; 5 years from Vineland, NJ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Oracle -&gt; Nvidia purchase $40bn</t>
+          <t>Microsoft -&gt; Nebius purchase $19.4bn; Nebius -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3350,12 +3348,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3365,43 +3363,47 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://nebius.com/newsroom/nebius-announces-multi-billion-dollar-agreement-with-microsoft-for-ai-infrastructure</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2025-05-14</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>OpenAI expands CoreWeave contract by $4bn</t>
+          <t>Nvidia agrees $1.5bn to rent back its own GPUs from Lambda</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
-      </c>
-      <c r="D61" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>$1.3bn for 10,000 GPUs + $200m for 8,000 (The Information)</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; CoreWeave purchase $4bn</t>
+          <t>Nvidia -&gt; Lambda backstop $1.5bn; Lambda -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3411,37 +3413,37 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://www.theinformation.com/articles/nvidia-quietly-boosts-cloud-ally-1-5-billion-deal-rent-ai-chips</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2025-03-31</t>
+          <t>2025-08-14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>OpenAI raises $40bn led by SoftBank at a $300bn valuation</t>
+          <t>Google backstops $3.2bn of Fluidstack leases at TeraWulf for a stake</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>40</v>
+        <v>6.9</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>SoftBank $30bn of $40bn; second $22.5bn tranche paid Dec 2025</t>
+          <t>Google takes warrants for ~14% of TeraWulf after the Sept expansion</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SoftBank -&gt; OpenAI investment $30bn</t>
+          <t>Google -&gt; Fluidstack backstop $3.2bn; TeraWulf -&gt; Google stock_grant; Fluidstack -&gt; TeraWulf purchase $3.7bn</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3461,43 +3463,47 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://openai.com/index/march-funding-updates/</t>
+          <t>https://investors.terawulf.com/news-events/press-releases</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2025-03-28</t>
+          <t>2025-07-22</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Nvidia anchors CoreWeave's IPO with a $250m order</t>
+          <t>OpenAI commits ~$300bn to Oracle for 4.5 GW of Stargate capacity</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D63" t="inlineStr"/>
+        <v>300</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>4.5 GW confirmed; ~$300bn over ~5 years from 2027 reported (WSJ)</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; CoreWeave investment $0.25bn; CoreWeave -&gt; Nvidia purchase</t>
+          <t>OpenAI -&gt; Oracle purchase $300bn</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3507,32 +3513,28 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://openai.com/index/stargate-advances-with-partnership-with-oracle/ | https://www.ft.com/content/86895a63-2c5b-4aea-b385-418130b64996</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-06-12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>OpenAI signs $11.9bn CoreWeave contract and takes $350m of CoreWeave stock</t>
+          <t>Meta buys 49% of Scale AI for $14.3bn</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>12.25</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>5-year contract</t>
-        </is>
-      </c>
+        <v>14.3</v>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OpenAI -&gt; CoreWeave purchase $11.9bn; OpenAI -&gt; CoreWeave investment $0.35bn</t>
+          <t>Meta -&gt; Scale AI investment $14.3bn; Meta -&gt; Scale AI purchase</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3557,47 +3559,47 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K | https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>2025-05-23</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SoftBank to spend $3bn a year on OpenAI tools (Cristal intelligence JV)</t>
+          <t>Oracle to buy ~$40bn of Nvidia chips for OpenAI's Abilene site</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>per year</t>
+          <t>~400,000 GB200s (FT)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SoftBank -&gt; OpenAI purchase $3bn</t>
+          <t>Oracle -&gt; Nvidia purchase $40bn</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>reported</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3607,42 +3609,38 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://group.softbank/en/news/press/20250203</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025-01-21</t>
+          <t>2025-05-14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Stargate: SoftBank, OpenAI, Oracle and MGX plan $500bn of US AI data centres</t>
+          <t>OpenAI expands CoreWeave contract by $4bn</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>500</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>4-year plan, $100bn 'immediately'; umbrella - not summed</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>SoftBank -&gt; Stargate investment; OpenAI -&gt; Stargate investment; Oracle -&gt; Stargate investment; MGX -&gt; Stargate investment; Stargate -&gt; Nvidia purchase</t>
+          <t>OpenAI -&gt; CoreWeave purchase $4bn</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>customer_finances_supplier</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3652,42 +3650,42 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://openai.com/index/announcing-the-stargate-project/</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2024-12-23</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>xAI raises $6bn with Nvidia and AMD as strategic investors</t>
+          <t>OpenAI raises $40bn led by SoftBank at a $300bn valuation</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Series C round total</t>
+          <t>SoftBank $30bn of $40bn; second $22.5bn tranche paid Dec 2025</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; SpaceX / xAI investment; AMD -&gt; SpaceX / xAI investment; SpaceX / xAI -&gt; Nvidia purchase</t>
+          <t>SoftBank -&gt; OpenAI investment $30bn</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3707,32 +3705,28 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://x.ai/news/series-c</t>
+          <t>https://openai.com/index/march-funding-updates/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2025-03-28</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Crusoe raises $600m with Nvidia participating</t>
+          <t>Nvidia anchors CoreWeave's IPO with a $250m order</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Series D round total</t>
-        </is>
-      </c>
+        <v>0.25</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Crusoe investment; Crusoe -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; CoreWeave investment $0.25bn; CoreWeave -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3747,7 +3741,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3757,37 +3751,37 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2024-12-02</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Nvidia joins $700m private placement in Nebius</t>
+          <t>OpenAI signs $11.9bn CoreWeave contract and takes $350m of CoreWeave stock</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.7</v>
+        <v>12.25</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>with Accel and Orbis</t>
+          <t>5-year contract</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Nebius investment; Nebius -&gt; Nvidia purchase</t>
+          <t>OpenAI -&gt; CoreWeave purchase $11.9bn; OpenAI -&gt; CoreWeave investment $0.35bn</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3807,32 +3801,32 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://nebius.com/newsroom</t>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K | https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Amazon invests another $4bn in Anthropic; AWS primary training partner</t>
+          <t>SoftBank to spend $3bn a year on OpenAI tools (Cristal intelligence JV)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>total Amazon investment $8bn</t>
+          <t>per year</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Amazon -&gt; Anthropic investment $4bn; Anthropic -&gt; Amazon purchase</t>
+          <t>SoftBank -&gt; OpenAI purchase $3bn</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3842,7 +3836,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>announced</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3857,32 +3851,32 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/anthropic-amazon-trainium</t>
+          <t>https://group.softbank/en/news/press/20250203</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>2025-01-21</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>OpenAI raises $6.6bn; Microsoft, Nvidia and SoftBank join</t>
+          <t>Stargate: SoftBank, OpenAI, Oracle and MGX plan $500bn of US AI data centres</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>6.6</v>
+        <v>500</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>round total at $157bn valuation; strategic pieces reported</t>
+          <t>4-year plan, $100bn 'immediately'; umbrella - not summed</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; OpenAI investment $0.75bn; Nvidia -&gt; OpenAI investment $0.1bn; SoftBank -&gt; OpenAI investment $0.5bn; OpenAI -&gt; Microsoft purchase</t>
+          <t>SoftBank -&gt; Stargate investment; OpenAI -&gt; Stargate investment; Oracle -&gt; Stargate investment; MGX -&gt; Stargate investment; Stargate -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3892,52 +3886,52 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>conditional</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://openai.com/index/scale-the-benefits-of-ai/</t>
+          <t>https://openai.com/index/announcing-the-stargate-project/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>2024-12-23</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Google pays ~$2.7bn to license Character.AI and rehire its founders</t>
+          <t>xAI raises $6bn with Nvidia and AMD as strategic investors</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2.7</v>
+        <v>6</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>reported (WSJ)</t>
+          <t>Series C round total</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Google -&gt; Character.AI licensing $2.7bn; Character.AI -&gt; Google purchase</t>
+          <t>Nvidia -&gt; SpaceX / xAI investment; AMD -&gt; SpaceX / xAI investment; SpaceX / xAI -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3947,7 +3941,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3957,37 +3951,37 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://x.ai/news/series-c</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2024-05-21</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Scale AI raises $1bn from Amazon, Meta, Nvidia and others</t>
+          <t>Crusoe raises $600m with Nvidia participating</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>round total</t>
+          <t>Series D round total</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Scale AI investment; Amazon -&gt; Scale AI investment; Meta -&gt; Scale AI investment; Meta -&gt; Scale AI purchase</t>
+          <t>Nvidia -&gt; Crusoe investment; Crusoe -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3997,7 +3991,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4007,33 +4001,37 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://scale.com/blog/scale-ai-series-f</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2024-04-16</t>
+          <t>2024-12-02</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Microsoft invests $1.5bn in G42; G42 runs on Azure</t>
+          <t>Nvidia joins $700m private placement in Nebius</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D74" t="inlineStr"/>
+        <v>0.7</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>with Accel and Orbis</t>
+        </is>
+      </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; G42 investment $1.5bn; G42 -&gt; Microsoft purchase</t>
+          <t>Nvidia -&gt; Nebius investment; Nebius -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4053,32 +4051,32 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://nebius.com/newsroom</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2024-03-19</t>
+          <t>2024-11-22</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Microsoft pays Inflection ~$650m to license models and hire staff</t>
+          <t>Amazon invests another $4bn in Anthropic; AWS primary training partner</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.65</v>
+        <v>4</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>reported; repaid Inflection's investors</t>
+          <t>total Amazon investment $8bn</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Inflection AI licensing $0.65bn</t>
+          <t>Amazon -&gt; Anthropic investment $4bn; Anthropic -&gt; Amazon purchase</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4093,7 +4091,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4103,32 +4101,32 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.reuters.com/technology/microsoft-pay-inflection-ai-650-million-after-scooping-up-most-staff-source-says-2024-03-21/</t>
+          <t>https://www.anthropic.com/news/anthropic-amazon-trainium</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2024-02-29</t>
+          <t>2024-10-02</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Figure AI raises $675m from Microsoft, Nvidia, Intel and OpenAI fund</t>
+          <t>OpenAI raises $6.6bn; Microsoft, Nvidia and SoftBank join</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.675</v>
+        <v>6.6</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>round total</t>
+          <t>round total at $157bn valuation; strategic pieces reported</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Figure AI investment; Nvidia -&gt; Figure AI investment; Intel -&gt; Figure AI investment; OpenAI -&gt; Figure AI investment; Figure AI -&gt; Microsoft purchase</t>
+          <t>Microsoft -&gt; OpenAI investment $0.75bn; Nvidia -&gt; OpenAI investment $0.1bn; SoftBank -&gt; OpenAI investment $0.5bn; OpenAI -&gt; Microsoft purchase</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4143,7 +4141,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4153,32 +4151,32 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://openai.com/index/scale-the-benefits-of-ai/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2024-02-26</t>
+          <t>2024-08-02</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Microsoft takes small stake in Mistral; models go on Azure</t>
+          <t>Google pays ~$2.7bn to license Character.AI and rehire its founders</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.016</v>
+        <v>2.7</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>EUR15m convertible</t>
+          <t>reported (WSJ)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Mistral investment $0.02bn; Mistral -&gt; Microsoft purchase</t>
+          <t>Google -&gt; Character.AI licensing $2.7bn; Character.AI -&gt; Google purchase</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4193,7 +4191,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4210,16 +4208,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
+          <t>2024-05-21</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Lambda raises $320m Series C with Nvidia</t>
+          <t>Scale AI raises $1bn from Amazon, Meta, Nvidia and others</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.32</v>
+        <v>1</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -4228,12 +4226,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Lambda investment; Lambda -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; Scale AI investment; Amazon -&gt; Scale AI investment; Meta -&gt; Scale AI investment; Meta -&gt; Scale AI purchase</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4253,37 +4251,33 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>https://lambdalabs.com/blog/lambda-raises-320m-to-build-a-gpu-cloud-for-ai</t>
+          <t>https://scale.com/blog/scale-ai-series-f</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2023-12-10</t>
+          <t>2024-04-16</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Mistral raises EUR385m Series A with Nvidia and Salesforce</t>
+          <t>Microsoft invests $1.5bn in G42; G42 runs on Azure</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.415</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>EUR385m at ~1.08 USD</t>
-        </is>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Mistral investment; Mistral -&gt; Nvidia purchase</t>
+          <t>Microsoft -&gt; G42 investment $1.5bn; G42 -&gt; Microsoft purchase</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4293,7 +4287,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4310,25 +4304,25 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2023-10-27</t>
+          <t>2024-03-19</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Google agrees to invest up to $2bn in Anthropic</t>
+          <t>Microsoft pays Inflection ~$650m to license models and hire staff</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>5</v>
+        <v>0.65</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>$500m upfront, $1.5bn over time; plus a multi-year Google Cloud deal reported at &gt;$3bn</t>
+          <t>reported; repaid Inflection's investors</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Google -&gt; Anthropic investment $2bn; Anthropic -&gt; Google purchase $3bn</t>
+          <t>Microsoft -&gt; Inflection AI licensing $0.65bn</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4338,7 +4332,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>reported</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4353,32 +4347,32 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>https://www.reuters.com/technology/google-agrees-invest-up-2-bln-openai-rival-anthropic-wsj-2023-10-27/</t>
+          <t>https://www.reuters.com/technology/microsoft-pay-inflection-ai-650-million-after-scooping-up-most-staff-source-says-2024-03-21/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2023-09-25</t>
+          <t>2024-02-29</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Amazon to invest up to $4bn in Anthropic; AWS becomes primary cloud</t>
+          <t>Figure AI raises $675m from Microsoft, Nvidia, Intel and OpenAI fund</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>0.675</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>$1.25bn initially, completed with $2.75bn in Mar 2024</t>
+          <t>round total</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Amazon -&gt; Anthropic investment $4bn; Anthropic -&gt; Amazon purchase</t>
+          <t>Microsoft -&gt; Figure AI investment; Nvidia -&gt; Figure AI investment; Intel -&gt; Figure AI investment; OpenAI -&gt; Figure AI investment; Figure AI -&gt; Microsoft purchase</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4403,32 +4397,32 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>https://www.aboutamazon.com/news/company-news/amazon-aws-anthropic-ai</t>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2023-08-24</t>
+          <t>2024-02-26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Hugging Face raises $235m from Google, Amazon, Nvidia, AMD, Intel and Salesforce</t>
+          <t>Microsoft takes small stake in Mistral; models go on Azure</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.235</v>
+        <v>0.016</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>round total</t>
+          <t>EUR15m convertible</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Hugging Face investment; Amazon -&gt; Hugging Face investment; Google -&gt; Hugging Face investment; AMD -&gt; Hugging Face investment; Intel -&gt; Hugging Face investment; Hugging Face -&gt; Amazon purchase</t>
+          <t>Microsoft -&gt; Mistral investment $0.02bn; Mistral -&gt; Microsoft purchase</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4460,16 +4454,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2023-06-29</t>
+          <t>2024-02-15</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Inflection AI raises $1.3bn from Microsoft and Nvidia, builds 22,000-H100 cluster</t>
+          <t>Lambda raises $320m Series C with Nvidia</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.3</v>
+        <v>0.32</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -4478,7 +4472,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; Inflection AI investment; Nvidia -&gt; Inflection AI investment; Inflection AI -&gt; CoreWeave purchase; CoreWeave -&gt; Nvidia purchase</t>
+          <t>Nvidia -&gt; Lambda investment; Lambda -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4503,37 +4497,37 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+          <t>https://lambdalabs.com/blog/lambda-raises-320m-to-build-a-gpu-cloud-for-ai</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-12-10</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Cohere raises $270m from Nvidia, Oracle and Salesforce</t>
+          <t>Mistral raises EUR385m Series A with Nvidia and Salesforce</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.27</v>
+        <v>0.415</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>round total</t>
+          <t>EUR385m at ~1.08 USD</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; Cohere investment; Oracle -&gt; Cohere investment; Cohere -&gt; Oracle purchase</t>
+          <t>Nvidia -&gt; Mistral investment; Mistral -&gt; Nvidia purchase</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>investor_is_counterparty</t>
+          <t>supplier_finances_customer</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4543,7 +4537,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4560,30 +4554,30 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2023-06-01</t>
+          <t>2023-10-27</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Microsoft signs multibillion GPU-capacity contracts with CoreWeave</t>
+          <t>Google agrees to invest up to $2bn in Anthropic</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>~$10bn through 2030 (reported); terms undisclosed</t>
+          <t>$500m upfront, $1.5bn over time; plus a multi-year Google Cloud deal reported at &gt;$3bn</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Microsoft -&gt; CoreWeave purchase $10bn</t>
+          <t>Google -&gt; Anthropic investment $2bn; Anthropic -&gt; Google purchase $3bn</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>customer_finances_supplier</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4603,37 +4597,37 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>https://www.cnbc.com/2023/06/01/microsoft-inks-deal-with-coreweave-to-meet-openai-cloud-demand.html</t>
+          <t>https://www.reuters.com/technology/google-agrees-invest-up-2-bln-openai-rival-anthropic-wsj-2023-10-27/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2023-04-20</t>
+          <t>2023-09-25</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nvidia joins CoreWeave's $221m round; H100s later collateralise $2.3bn debt</t>
+          <t>Amazon to invest up to $4bn in Anthropic; AWS becomes primary cloud</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.221</v>
+        <v>4</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Series B extension; Aug-2023 $2.3bn debt facility secured on Nvidia GPUs</t>
+          <t>$1.25bn initially, completed with $2.75bn in Mar 2024</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Nvidia -&gt; CoreWeave investment; CoreWeave -&gt; Nvidia purchase</t>
+          <t>Amazon -&gt; Anthropic investment $4bn; Anthropic -&gt; Amazon purchase</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>supplier_finances_customer</t>
+          <t>investor_is_counterparty</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4653,55 +4647,305 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+          <t>https://www.aboutamazon.com/news/company-news/amazon-aws-anthropic-ai</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>2023-08-24</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Hugging Face raises $235m from Google, Amazon, Nvidia, AMD, Intel and Salesforce</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>round total</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Nvidia -&gt; Hugging Face investment; Amazon -&gt; Hugging Face investment; Google -&gt; Hugging Face investment; AMD -&gt; Hugging Face investment; Intel -&gt; Hugging Face investment; Hugging Face -&gt; Amazon purchase</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>investor_is_counterparty</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2023-06-29</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Inflection AI raises $1.3bn from Microsoft and Nvidia, builds 22,000-H100 cluster</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>round total</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Microsoft -&gt; Inflection AI investment; Nvidia -&gt; Inflection AI investment; Inflection AI -&gt; CoreWeave purchase; CoreWeave -&gt; Nvidia purchase</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2023-06-08</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Cohere raises $270m from Nvidia, Oracle and Salesforce</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>round total</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Nvidia -&gt; Cohere investment; Oracle -&gt; Cohere investment; Cohere -&gt; Oracle purchase</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>investor_is_counterparty</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/8475dc9b-b2d4-4e10-a6b6-12796b11758a</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2023-06-01</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Microsoft signs multibillion GPU-capacity contracts with CoreWeave</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>10</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>~$10bn through 2030 (reported); terms undisclosed</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Microsoft -&gt; CoreWeave purchase $10bn</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>customer_finances_supplier</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2023/06/01/microsoft-inks-deal-with-coreweave-to-meet-openai-cloud-demand.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2023-04-20</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Nvidia joins CoreWeave's $221m round; H100s later collateralise $2.3bn debt</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Series B extension; Aug-2023 $2.3bn debt facility secured on Nvidia GPUs</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Nvidia -&gt; CoreWeave investment; CoreWeave -&gt; Nvidia purchase</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001769628&amp;type=8-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>2023-01-23</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>Microsoft extends OpenAI partnership (~$10bn)</t>
         </is>
       </c>
-      <c r="C87" t="n">
+      <c r="C92" t="n">
         <v>10</v>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>multiyear, multibillion; $10bn widely reported, not confirmed by Microsoft</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>Microsoft -&gt; OpenAI investment $10bn; OpenAI -&gt; Microsoft purchase</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>investor_is_counterparty</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
+      <c r="G92" t="inlineStr">
         <is>
           <t>closed</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
+      <c r="I92" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="J92" t="inlineStr">
         <is>
           <t>https://blogs.microsoft.com/blog/2023/01/23/microsoftandopenaiextendpartnership/</t>
         </is>
@@ -4718,7 +4962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O175"/>
+  <dimension ref="A1:O183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -12371,7 +12615,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>paid in full</t>
+          <t>paid in three $10bn tranches; last on 1 Oct 2026 (SoftBank total ~$64.6bn, ~13%)</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -14852,6 +15096,413 @@
       <c r="N175" t="inlineStr">
         <is>
           <t>2025-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>nscale-figure-2026-09</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Nscale sells Figure AI $3.5bn of compute and takes an equity stake</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Figure AI</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>investment</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>undisclosed strategic stake; Nscale becomes preferred compute provider</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>nscale-figure-2026-09</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Nscale sells Figure AI $3.5bn of compute and takes an equity stake</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Figure AI</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="G177" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>up to 100k Nvidia Vera Rubin GPUs in Barstow TX from H2 2027</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>qcom-amzn-2026-09</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Qualcomm gives Amazon warrants worth up to $4bn tied to AI data-centre chip purchases</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Qualcomm</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>stock_grant</t>
+        </is>
+      </c>
+      <c r="G178" t="n">
+        <v>4</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>warrant for 25m Qualcomm shares, vests with purchases</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>716.92</v>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="O178" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>qcom-amzn-2026-09</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Qualcomm gives Amazon warrants worth up to $4bn tied to AI data-centre chip purchases</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Qualcomm</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>custom inference chips + optical interconnects; vesting ceiling $60bn</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>supplier_finances_customer</t>
+        </is>
+      </c>
+      <c r="J179" t="n">
+        <v>716.92</v>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>nvda-figure-2026-10</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Nvidia discusses investing another $1bn in Figure AI</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Figure AI</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>investment</t>
+        </is>
+      </c>
+      <c r="G180" t="n">
+        <v>1</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>talks; Nvidia already an investor and Figure's GPU supplier</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>investor_is_counterparty</t>
+        </is>
+      </c>
+      <c r="J180" t="n">
+        <v>215.94</v>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>nvda-reflection-2026-10</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Nvidia in talks to deepen its Reflection AI stake, supply more chips, or buy it</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Reflection AI</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>investment</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>larger stake, acqui-hire or acquisition under discussion</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>investor_is_counterparty</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v>215.94</v>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>nvda-reflection-2026-10</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Nvidia in talks to deepen its Reflection AI stake, supply more chips, or buy it</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Reflection AI</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>additional chip supply under discussion</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>investor_is_counterparty</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>215.94</v>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>anthropic-iren-2026-10</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Anthropic signs an unannounced multiyear cloud deal with Nvidia-backed IREN</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>multiyear AI cloud contract (likely the unnamed frontier-lab deal IREN flagged in Aug)</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>customer_finances_supplier</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>

</xml_diff>